<commit_message>
Update Kahoot Change-or-Go-Under questions to bilingual EN-ZH
</commit_message>
<xml_diff>
--- a/change-or-go-under-quiz/Kahoot-Change-or-Go-Under.xlsx
+++ b/change-or-go-under-quiz/Kahoot-Change-or-Go-Under.xlsx
@@ -707,7 +707,7 @@
       </c>
       <c r="B9" s="22" t="inlineStr">
         <is>
-          <t>What causes sea levels to rise around the world?</t>
+          <t>What causes sea levels to rise around the world? 什麼導致海平面上升?</t>
         </is>
       </c>
       <c r="C9" s="22" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="B10" s="25" t="inlineStr">
         <is>
-          <t>Why are people's lives in danger?</t>
+          <t>Why are people's lives in danger? 為什麼人們的生活陷入危險?</t>
         </is>
       </c>
       <c r="C10" s="25" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="B11" s="25" t="inlineStr">
         <is>
-          <t>Where did people on a small island in Panama move?</t>
+          <t>Where did people on a small island in Panama move? 巴拿馬小島居民搬到哪?</t>
         </is>
       </c>
       <c r="C11" s="25" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
-          <t>In Panama, many fishermen became ___.</t>
+          <t>In Panama, many fishermen became ___. 在巴拿馬,漁夫變成了___?</t>
         </is>
       </c>
       <c r="C12" s="25" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>What are people designing in the Maldives?</t>
+          <t>What are people designing in the Maldives? 馬爾地夫正在設計什麼?</t>
         </is>
       </c>
       <c r="C13" s="25" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="B14" s="25" t="inlineStr">
         <is>
-          <t>The Maldives floating city can also ___ sea life.</t>
+          <t>The Maldives floating city can also ___ sea life. 漂浮城市還能___海洋生物?</t>
         </is>
       </c>
       <c r="C14" s="25" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="B15" s="25" t="inlineStr">
         <is>
-          <t>The Maldives city works with ___ and may never go under.</t>
+          <t>The Maldives city works with ___ and may never go under. 這城市與___合作而不沉沒?</t>
         </is>
       </c>
       <c r="C15" s="25" t="inlineStr">
@@ -980,7 +980,7 @@
       </c>
       <c r="B16" s="25" t="inlineStr">
         <is>
-          <t>What is the Reading Skill in this lesson?</t>
+          <t>What is the Reading Skill in this lesson? 本課的閱讀策略是什麼?</t>
         </is>
       </c>
       <c r="C16" s="25" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="B17" s="25" t="inlineStr">
         <is>
-          <t>Taiwan is an island, too. What should we do?</t>
+          <t>Taiwan is an island, too. What should we do? 台灣也是島嶼,我們該怎麼做?</t>
         </is>
       </c>
       <c r="C17" s="25" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="B18" s="25" t="inlineStr">
         <is>
-          <t>fishermen is the plural form of which word?</t>
+          <t>fishermen is the plural form of which word? fishermen是哪個字的複數?</t>
         </is>
       </c>
       <c r="C18" s="25" t="inlineStr">

</xml_diff>